<commit_message>
Format output as  Part 1 & 2
</commit_message>
<xml_diff>
--- a/static/marks_template.xlsx
+++ b/static/marks_template.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -28,7 +28,7 @@
     <t xml:space="preserve">Name</t>
   </si>
   <si>
-    <t xml:space="preserve">Test1_CO1</t>
+    <t xml:space="preserve">Test_CO1</t>
   </si>
   <si>
     <t xml:space="preserve">Assign_CO1</t>

</xml_diff>